<commit_message>
extra notes for zybooks
</commit_message>
<xml_diff>
--- a/Lab3Analysis/results.xlsx
+++ b/Lab3Analysis/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\COP3503C\Lab3Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB1F545A-56F1-4E76-B4C0-41EB81D347AC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0551BD31-22D6-4099-8AA6-2E40D4AEC996}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{5F0913F3-B6AB-45BE-945A-6C3D7068312E}"/>
   </bookViews>
@@ -20,24 +20,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">results!$A$1:$E$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="25">
   <si>
     <t>Task</t>
   </si>
@@ -109,6 +96,9 @@
   </si>
   <si>
     <t>ABQ Scale Factor 2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -4423,19 +4413,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.15773999999999999</c:v>
+                  <c:v>0.18937399999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.43924600000000003</c:v>
+                  <c:v>0.59200299999999995</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.72861399999999998</c:v>
+                  <c:v>0.92942999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.2102999999999999</c:v>
+                  <c:v>1.37951</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.4164000000000001</c:v>
+                  <c:v>1.9923999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4504,19 +4494,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.15831799999999999</c:v>
+                  <c:v>0.19003100000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.48785099999999998</c:v>
+                  <c:v>0.59532300000000005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.729217</c:v>
+                  <c:v>0.93585799999999997</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.2423200000000001</c:v>
+                  <c:v>1.3950899999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.4371700000000001</c:v>
+                  <c:v>1.9825999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14688,7 +14678,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BF0C1F-A754-415C-A443-CE584771C95E}">
-  <dimension ref="A1:C150"/>
+  <dimension ref="A1:D150"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="3" width="10" bestFit="1" customWidth="1"/>
@@ -14774,7 +14764,7 @@
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -14785,7 +14775,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:4">
       <c r="A18">
         <v>10000000</v>
       </c>
@@ -14796,7 +14786,7 @@
         <v>0.144261</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:4">
       <c r="A19">
         <v>30000000</v>
       </c>
@@ -14807,7 +14797,7 @@
         <v>0.36504700000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:4">
       <c r="A20">
         <v>50000000</v>
       </c>
@@ -14818,7 +14808,7 @@
         <v>0.705183</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:4">
       <c r="A21">
         <v>75000000</v>
       </c>
@@ -14829,7 +14819,7 @@
         <v>1.11677</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:4">
       <c r="A22">
         <v>100000000</v>
       </c>
@@ -14840,7 +14830,12 @@
         <v>1.3060799999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="24" spans="1:4">
+      <c r="D24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="1" t="s">
         <v>16</v>
       </c>
@@ -15082,10 +15077,10 @@
         <v>10000000</v>
       </c>
       <c r="B82">
-        <v>0.15773999999999999</v>
+        <v>0.18937399999999999</v>
       </c>
       <c r="C82">
-        <v>0.15831799999999999</v>
+        <v>0.19003100000000001</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -15093,10 +15088,10 @@
         <v>30000000</v>
       </c>
       <c r="B83">
-        <v>0.43924600000000003</v>
+        <v>0.59200299999999995</v>
       </c>
       <c r="C83">
-        <v>0.48785099999999998</v>
+        <v>0.59532300000000005</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -15104,10 +15099,10 @@
         <v>50000000</v>
       </c>
       <c r="B84">
-        <v>0.72861399999999998</v>
+        <v>0.92942999999999998</v>
       </c>
       <c r="C84">
-        <v>0.729217</v>
+        <v>0.93585799999999997</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -15115,10 +15110,10 @@
         <v>75000000</v>
       </c>
       <c r="B85">
-        <v>1.2102999999999999</v>
+        <v>1.37951</v>
       </c>
       <c r="C85">
-        <v>1.2423200000000001</v>
+        <v>1.3950899999999999</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -15126,10 +15121,10 @@
         <v>100000000</v>
       </c>
       <c r="B86">
-        <v>1.4164000000000001</v>
+        <v>1.9923999999999999</v>
       </c>
       <c r="C86">
-        <v>1.4371700000000001</v>
+        <v>1.9825999999999999</v>
       </c>
     </row>
     <row r="96" spans="1:3">

</xml_diff>